<commit_message>
Add SD card and transforms documentation, update to-do list
</commit_message>
<xml_diff>
--- a/To do/To do list.xlsx
+++ b/To do/To do list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\BODAQS\To do\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FBDD51F6-7CDB-4F56-B5F0-A84067A38E7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4579204B-08F4-49BF-94C9-D962A20BC6BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="360" windowWidth="25845" windowHeight="15120" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="15720" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
   </bookViews>
   <sheets>
     <sheet name="ToDo" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="Stripboard (2)" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="178">
   <si>
     <t>Requirements</t>
   </si>
@@ -562,6 +563,21 @@
   </si>
   <si>
     <t>Think about connector style and location</t>
+  </si>
+  <si>
+    <t>Drop option for zeroed column</t>
+  </si>
+  <si>
+    <t>Invert behaviour, in relation to zero / full range</t>
+  </si>
+  <si>
+    <t>Only connect if RTC isn't set</t>
+  </si>
+  <si>
+    <t>save/cancel menu on calibration</t>
+  </si>
+  <si>
+    <t>Draining to dedicated storage task</t>
   </si>
 </sst>
 </file>
@@ -6934,10 +6950,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7574,6 +7586,21 @@
         <v>157</v>
       </c>
     </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>176</v>
+      </c>
+    </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="13" t="s">
         <v>159</v>
@@ -7583,6 +7610,9 @@
       <c r="A56" s="1" t="s">
         <v>160</v>
       </c>
+      <c r="C56" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
@@ -7637,6 +7667,9 @@
       <c r="C66" s="1"/>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>177</v>
+      </c>
       <c r="C67" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Make zeroing optional and geberate a mask for inactive sections
</commit_message>
<xml_diff>
--- a/To do/To do list.xlsx
+++ b/To do/To do list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\BODAQS\To do\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA905A05-904F-4ABF-8465-A26DD2EE3FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{642B9AD6-85C9-48D7-81FD-718C808568B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="360" windowWidth="25845" windowHeight="15120" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="32070" windowHeight="15120" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
   </bookViews>
   <sheets>
     <sheet name="ToDo" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="177">
   <si>
     <t>Requirements</t>
   </si>
@@ -387,9 +387,6 @@
     <t>data_active_rs</t>
   </si>
   <si>
-    <t>Continue config cleanup</t>
-  </si>
-  <si>
     <t>Firmware</t>
   </si>
   <si>
@@ -402,9 +399,6 @@
     <t>Do some basic bike setup record keeping</t>
   </si>
   <si>
-    <t>Fix funny 'raw' columns</t>
-  </si>
-  <si>
     <t>Expand to accelerometers</t>
   </si>
   <si>
@@ -414,9 +408,6 @@
     <t>Big code cleanup, refactor and document</t>
   </si>
   <si>
-    <t>Rebound analysis refactor / generalise</t>
-  </si>
-  <si>
     <t>Mechanical</t>
   </si>
   <si>
@@ -432,9 +423,6 @@
     <t>Build accelerometer mount</t>
   </si>
   <si>
-    <t>Brainstorm test cases</t>
-  </si>
-  <si>
     <t>Sensor re-factor and individual sample rate</t>
   </si>
   <si>
@@ -583,6 +571,9 @@
   </si>
   <si>
     <t>Domains derived from some master source</t>
+  </si>
+  <si>
+    <t>Pass activity-mask parameters from notebook</t>
   </si>
 </sst>
 </file>
@@ -7449,16 +7440,16 @@
     <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="C27" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="E27" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="E27" s="13" t="s">
-        <v>117</v>
-      </c>
       <c r="G27" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -7470,32 +7461,26 @@
         <v>98</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E29" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>95</v>
       </c>
-      <c r="C30" t="s">
-        <v>129</v>
-      </c>
       <c r="E30" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>96</v>
       </c>
-      <c r="C31" t="s">
-        <v>114</v>
-      </c>
       <c r="E31" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -7503,50 +7488,47 @@
         <v>97</v>
       </c>
       <c r="C32" t="s">
-        <v>119</v>
+        <v>176</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C33" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E33" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="E34" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C35" s="1"/>
       <c r="E35" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -7554,114 +7536,114 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="16" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="E44" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E45" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E46" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="13" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="13" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C61" s="1"/>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C62" s="1"/>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C63" s="1"/>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C65" s="1"/>
     </row>
@@ -7670,23 +7652,23 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C67" s="1"/>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -7753,10 +7735,10 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -7923,21 +7905,21 @@
   <sheetData>
     <row r="4" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E4" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="G4" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="I4" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E5" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="F5" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -7946,13 +7928,13 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="L5" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="M5" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" spans="5:13" x14ac:dyDescent="0.25">
@@ -7960,7 +7942,7 @@
         <v>70</v>
       </c>
       <c r="F6" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="G6">
         <v>2</v>
@@ -7969,18 +7951,18 @@
         <v>2</v>
       </c>
       <c r="J6" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="L6" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="M6" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="F7" t="s">
         <v>83</v>
@@ -7992,21 +7974,21 @@
         <v>3</v>
       </c>
       <c r="J7" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="L7" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="M7" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8" spans="5:13" x14ac:dyDescent="0.25">
       <c r="L8" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="M8" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Consumer side: develop a session selector and convert two widgets - signal histogram and event browser - to use it. Re-factor the event browser to remove redundant UI elements and improve what remains.
</commit_message>
<xml_diff>
--- a/To do/To do list.xlsx
+++ b/To do/To do list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\BODAQS\To do\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{642B9AD6-85C9-48D7-81FD-718C808568B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30B0C306-BF07-400B-BDCB-29343F53EAEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="32070" windowHeight="15120" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
+    <workbookView xWindow="1170" yWindow="1080" windowWidth="18210" windowHeight="15120" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
   </bookViews>
   <sheets>
     <sheet name="ToDo" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="178">
   <si>
     <t>Requirements</t>
   </si>
@@ -574,6 +574,9 @@
   </si>
   <si>
     <t>Pass activity-mask parameters from notebook</t>
+  </si>
+  <si>
+    <t>Pre-processing fails if zeroing is false</t>
   </si>
 </sst>
 </file>
@@ -7495,6 +7498,9 @@
       <c r="A33" s="3" t="s">
         <v>126</v>
       </c>
+      <c r="C33" t="s">
+        <v>177</v>
+      </c>
       <c r="E33" t="s">
         <v>166</v>
       </c>

</xml_diff>

<commit_message>
Implement rebuild of widgets if session selector changes. Migrate metrics histogram widget. Cosmetic changes to widget layouts.
</commit_message>
<xml_diff>
--- a/To do/To do list.xlsx
+++ b/To do/To do list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\BODAQS\To do\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30B0C306-BF07-400B-BDCB-29343F53EAEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC7BECB-B789-4509-B957-9F9E4A3FA67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1080" windowWidth="18210" windowHeight="15120" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
+    <workbookView xWindow="3615" yWindow="180" windowWidth="18210" windowHeight="15120" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
   </bookViews>
   <sheets>
     <sheet name="ToDo" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="183">
   <si>
     <t>Requirements</t>
   </si>
@@ -577,6 +577,21 @@
   </si>
   <si>
     <t>Pre-processing fails if zeroing is false</t>
+  </si>
+  <si>
+    <t>Widgets - option to display sessions by description</t>
+  </si>
+  <si>
+    <t>Widgets - order signals by unit</t>
+  </si>
+  <si>
+    <t>Metrics scatter - cosmetics</t>
+  </si>
+  <si>
+    <t>Metrics scatter - sensor / signal more sensible</t>
+  </si>
+  <si>
+    <t>Metrics histogram - stats optional</t>
   </si>
 </sst>
 </file>
@@ -7526,15 +7541,34 @@
       <c r="A36" t="s">
         <v>119</v>
       </c>
+      <c r="C36" t="s">
+        <v>178</v>
+      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>120</v>
       </c>
+      <c r="C37" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C38" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C39" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>154</v>
+      </c>
+      <c r="C40" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Finish cosmetic tidy up of widgets. Stop inferring sensors from signal names and use the registry and schema instead.
</commit_message>
<xml_diff>
--- a/To do/To do list.xlsx
+++ b/To do/To do list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\BODAQS\To do\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC7BECB-B789-4509-B957-9F9E4A3FA67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D6F278-1144-49E4-90D4-D104EC11FA1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3615" yWindow="180" windowWidth="18210" windowHeight="15120" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="182">
   <si>
     <t>Requirements</t>
   </si>
@@ -585,13 +585,10 @@
     <t>Widgets - order signals by unit</t>
   </si>
   <si>
-    <t>Metrics scatter - cosmetics</t>
-  </si>
-  <si>
-    <t>Metrics scatter - sensor / signal more sensible</t>
-  </si>
-  <si>
     <t>Metrics histogram - stats optional</t>
+  </si>
+  <si>
+    <t>Widgets - more useful default values</t>
   </si>
 </sst>
 </file>
@@ -7555,20 +7552,17 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C38" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C39" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>154</v>
-      </c>
-      <c r="C40" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Initial prototype of session browser widget
</commit_message>
<xml_diff>
--- a/To do/To do list.xlsx
+++ b/To do/To do list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\BODAQS\To do\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D6F278-1144-49E4-90D4-D104EC11FA1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8028C690-5084-4206-951F-1D74266A2AEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3615" yWindow="180" windowWidth="18210" windowHeight="15120" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="180">
   <si>
     <t>Requirements</t>
   </si>
@@ -582,13 +582,7 @@
     <t>Widgets - option to display sessions by description</t>
   </si>
   <si>
-    <t>Widgets - order signals by unit</t>
-  </si>
-  <si>
-    <t>Metrics histogram - stats optional</t>
-  </si>
-  <si>
-    <t>Widgets - more useful default values</t>
+    <t>Signal histogram widget: more elaborate detection of available signals</t>
   </si>
 </sst>
 </file>
@@ -7550,16 +7544,6 @@
         <v>179</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C38" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C39" t="s">
-        <v>180</v>
-      </c>
-    </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>154</v>

</xml_diff>

<commit_message>
Move session window browser to single-figure design and debug. Ready to commence managing marks and bookmarks
</commit_message>
<xml_diff>
--- a/To do/To do list.xlsx
+++ b/To do/To do list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\BODAQS\To do\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8028C690-5084-4206-951F-1D74266A2AEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F20A2001-C31D-4886-83FD-CCFE42702CE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3615" yWindow="180" windowWidth="18210" windowHeight="15120" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="183">
   <si>
     <t>Requirements</t>
   </si>
@@ -583,6 +583,15 @@
   </si>
   <si>
     <t>Signal histogram widget: more elaborate detection of available signals</t>
+  </si>
+  <si>
+    <t>Download all / delete all</t>
+  </si>
+  <si>
+    <t>Tidy up session window</t>
+  </si>
+  <si>
+    <t>Iterate event schema - all the events</t>
   </si>
 </sst>
 </file>
@@ -7274,7 +7283,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{939CC629-FF5C-4C16-8302-43E72468A454}">
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.28515625" bestFit="1" customWidth="1"/>
@@ -7548,9 +7557,15 @@
       <c r="A40" t="s">
         <v>154</v>
       </c>
+      <c r="C40" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
+      <c r="C41" t="s">
+        <v>182</v>
+      </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="16" t="s">
@@ -7687,6 +7702,11 @@
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>175</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update gitignore and todo
</commit_message>
<xml_diff>
--- a/To do/To do list.xlsx
+++ b/To do/To do list.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\BODAQS\To do\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benco\dev\BODAQS\To do\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA905A05-904F-4ABF-8465-A26DD2EE3FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94877A1A-BA37-4118-87CB-090657EE4E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="360" windowWidth="25845" windowHeight="15120" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
   </bookViews>
   <sheets>
     <sheet name="ToDo" sheetId="1" r:id="rId1"/>
-    <sheet name="ThingPlus" sheetId="8" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
-    <sheet name="PinOut" sheetId="3" r:id="rId4"/>
-    <sheet name="4_D pins" sheetId="10" r:id="rId5"/>
-    <sheet name="Stripboard" sheetId="5" r:id="rId6"/>
-    <sheet name="Dataframes" sheetId="6" r:id="rId7"/>
-    <sheet name="Stripboard (2)" sheetId="9" r:id="rId8"/>
+    <sheet name="Sheet1" sheetId="11" r:id="rId2"/>
+    <sheet name="ThingPlus" sheetId="8" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId4"/>
+    <sheet name="PinOut" sheetId="3" r:id="rId5"/>
+    <sheet name="4_D pins" sheetId="10" r:id="rId6"/>
+    <sheet name="Stripboard" sheetId="5" r:id="rId7"/>
+    <sheet name="Dataframes" sheetId="6" r:id="rId8"/>
+    <sheet name="Stripboard (2)" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="189">
   <si>
     <t>Requirements</t>
   </si>
@@ -339,9 +340,6 @@
     <t>AP mode</t>
   </si>
   <si>
-    <t>[mm]-&gt;_mm - column naming standard</t>
-  </si>
-  <si>
     <t>Load files</t>
   </si>
   <si>
@@ -387,9 +385,6 @@
     <t>data_active_rs</t>
   </si>
   <si>
-    <t>Continue config cleanup</t>
-  </si>
-  <si>
     <t>Firmware</t>
   </si>
   <si>
@@ -402,9 +397,6 @@
     <t>Do some basic bike setup record keeping</t>
   </si>
   <si>
-    <t>Fix funny 'raw' columns</t>
-  </si>
-  <si>
     <t>Expand to accelerometers</t>
   </si>
   <si>
@@ -414,9 +406,6 @@
     <t>Big code cleanup, refactor and document</t>
   </si>
   <si>
-    <t>Rebound analysis refactor / generalise</t>
-  </si>
-  <si>
     <t>Mechanical</t>
   </si>
   <si>
@@ -432,9 +421,6 @@
     <t>Build accelerometer mount</t>
   </si>
   <si>
-    <t>Brainstorm test cases</t>
-  </si>
-  <si>
     <t>Sensor re-factor and individual sample rate</t>
   </si>
   <si>
@@ -583,6 +569,48 @@
   </si>
   <si>
     <t>Domains derived from some master source</t>
+  </si>
+  <si>
+    <t>Pass activity-mask parameters from notebook</t>
+  </si>
+  <si>
+    <t>Pre-processing fails if zeroing is false</t>
+  </si>
+  <si>
+    <t>Widgets - option to display sessions by description</t>
+  </si>
+  <si>
+    <t>Signal histogram widget: more elaborate detection of available signals</t>
+  </si>
+  <si>
+    <t>Download all / delete all</t>
+  </si>
+  <si>
+    <t>Tidy up session window</t>
+  </si>
+  <si>
+    <t>Iterate event schema - all the events</t>
+  </si>
+  <si>
+    <t>Write NTP back to SD card</t>
+  </si>
+  <si>
+    <t>installed zeroes</t>
+  </si>
+  <si>
+    <t>front</t>
+  </si>
+  <si>
+    <t>rear</t>
+  </si>
+  <si>
+    <t>Don't zero in place</t>
+  </si>
+  <si>
+    <t>Pass zeroing parameters dynamically</t>
+  </si>
+  <si>
+    <t>Test clipping</t>
   </si>
 </sst>
 </file>
@@ -7274,22 +7302,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{939CC629-FF5C-4C16-8302-43E72468A454}">
-  <dimension ref="A1:G71"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G75"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="34.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5546875" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
-    <col min="5" max="5" width="39.28515625" customWidth="1"/>
+    <col min="5" max="5" width="39.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -7300,7 +7328,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
@@ -7308,7 +7336,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
         <v>8</v>
       </c>
@@ -7316,7 +7344,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>8</v>
       </c>
@@ -7324,8 +7352,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -7336,7 +7364,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>8</v>
       </c>
@@ -7344,10 +7372,10 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -7358,7 +7386,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
         <v>8</v>
       </c>
@@ -7366,7 +7394,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="B15" s="2" t="s">
         <v>8</v>
       </c>
@@ -7374,8 +7402,8 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>3</v>
       </c>
@@ -7386,7 +7414,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
         <v>6</v>
       </c>
@@ -7394,7 +7422,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B19" s="2" t="s">
         <v>8</v>
       </c>
@@ -7402,7 +7430,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B20" s="1" t="s">
         <v>6</v>
       </c>
@@ -7410,8 +7438,8 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>5</v>
       </c>
@@ -7422,7 +7450,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B23" s="2" t="s">
         <v>8</v>
       </c>
@@ -7430,7 +7458,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B24" s="2" t="s">
         <v>8</v>
       </c>
@@ -7438,7 +7466,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B25" s="2" t="s">
         <v>8</v>
       </c>
@@ -7446,247 +7474,273 @@
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="E27" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="C27" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="E27" s="13" t="s">
-        <v>117</v>
-      </c>
       <c r="G27" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="C28" s="1"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>98</v>
-      </c>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C29" s="15" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E29" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>95</v>
       </c>
-      <c r="C30" t="s">
-        <v>129</v>
-      </c>
       <c r="E30" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>96</v>
       </c>
-      <c r="C31" t="s">
-        <v>114</v>
-      </c>
       <c r="E31" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>97</v>
       </c>
-      <c r="C32" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C33" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E33" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E34" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C35" s="1"/>
       <c r="E35" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>118</v>
+      </c>
+      <c r="C36" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>119</v>
+      </c>
+      <c r="C37" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>153</v>
+      </c>
+      <c r="C40" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="1"/>
+      <c r="C41" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="16" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C43" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>131</v>
+      </c>
+      <c r="C44" t="s">
+        <v>186</v>
+      </c>
+      <c r="E44" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>132</v>
+      </c>
+      <c r="C45" t="s">
+        <v>187</v>
+      </c>
+      <c r="E45" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>133</v>
+      </c>
+      <c r="C46" t="s">
+        <v>175</v>
+      </c>
+      <c r="E46" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C47" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="13" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" s="13" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>160</v>
+      </c>
+      <c r="C61" s="1"/>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>161</v>
+      </c>
+      <c r="C62" s="1"/>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>162</v>
+      </c>
+      <c r="C63" s="1"/>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>163</v>
+      </c>
+      <c r="C65" s="1"/>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C66" s="1"/>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>171</v>
+      </c>
+      <c r="C67" s="1"/>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="1"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="16" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>136</v>
-      </c>
-      <c r="E44" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>137</v>
-      </c>
-      <c r="E45" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>138</v>
-      </c>
-      <c r="E46" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="13" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="s">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="13" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>165</v>
-      </c>
-      <c r="C61" s="1"/>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>166</v>
-      </c>
-      <c r="C62" s="1"/>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>167</v>
-      </c>
-      <c r="C63" s="1"/>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>168</v>
-      </c>
-      <c r="C65" s="1"/>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C66" s="1"/>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>176</v>
-      </c>
-      <c r="C67" s="1"/>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
         <v>179</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -7696,41 +7750,72 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1E285E6-E254-4E54-A2AD-B9383DD0CBCD}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B2">
+        <v>3433</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B3">
+        <v>3564</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{997F476F-FC8E-48EF-BCCB-17FEE9D854A7}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63A66E13-B34A-4CEF-9884-F713168D706E}">
   <dimension ref="A1:A11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>51</v>
       </c>
@@ -7742,24 +7827,24 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65146F67-0A23-4B02-A988-FD7EF72FDEF9}">
   <dimension ref="A1:I19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" customWidth="1"/>
-    <col min="2" max="2" width="8.140625" customWidth="1"/>
+    <col min="1" max="1" width="18.33203125" customWidth="1"/>
+    <col min="2" max="2" width="8.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C1" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="D1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>45</v>
       </c>
@@ -7767,7 +7852,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -7775,7 +7860,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -7786,7 +7871,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -7797,7 +7882,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>40</v>
       </c>
@@ -7808,7 +7893,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>41</v>
       </c>
@@ -7819,7 +7904,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>42</v>
       </c>
@@ -7830,7 +7915,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>43</v>
       </c>
@@ -7841,7 +7926,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -7849,7 +7934,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>46</v>
       </c>
@@ -7860,7 +7945,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>30</v>
       </c>
@@ -7871,7 +7956,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>29</v>
       </c>
@@ -7879,7 +7964,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>33</v>
       </c>
@@ -7887,7 +7972,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>34</v>
       </c>
@@ -7895,7 +7980,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>35</v>
       </c>
@@ -7903,7 +7988,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>36</v>
       </c>
@@ -7916,28 +8001,28 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6779A28B-13EE-492E-A8C9-A3EBA7018F9E}">
   <dimension ref="E4:M8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="4" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E4" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G4" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="I4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="5" spans="5:13" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="5" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E5" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="F5" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -7946,21 +8031,21 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="L5" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="M5" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="6" spans="5:13" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E6" t="s">
         <v>70</v>
       </c>
       <c r="F6" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="G6">
         <v>2</v>
@@ -7969,18 +8054,18 @@
         <v>2</v>
       </c>
       <c r="J6" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="L6" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="M6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="7" spans="5:13" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="7" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E7" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="F7" t="s">
         <v>83</v>
@@ -7992,21 +8077,21 @@
         <v>3</v>
       </c>
       <c r="J7" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="L7" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="M7" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="8" spans="5:13" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="8" spans="5:13" x14ac:dyDescent="0.3">
       <c r="L8" t="s">
+        <v>143</v>
+      </c>
+      <c r="M8" t="s">
         <v>148</v>
-      </c>
-      <c r="M8" t="s">
-        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -8015,27 +8100,27 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AD90B76-97FE-47FB-860F-1C66CC9E54CC}">
   <dimension ref="C3:BX43"/>
-  <sheetFormatPr defaultColWidth="2.7109375" defaultRowHeight="16.5" thickTop="1" thickBottom="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="2.6640625" defaultRowHeight="15.6" thickTop="1" thickBottom="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="2.7109375" style="6"/>
-    <col min="3" max="3" width="9.28515625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="5.28515625" style="4" customWidth="1"/>
-    <col min="5" max="7" width="2.7109375" style="4"/>
-    <col min="8" max="17" width="2.7109375" style="6"/>
-    <col min="18" max="18" width="7.5703125" style="6" customWidth="1"/>
-    <col min="19" max="46" width="2.7109375" style="6"/>
-    <col min="47" max="47" width="2.7109375" style="6" customWidth="1"/>
-    <col min="48" max="71" width="2.7109375" style="6"/>
-    <col min="72" max="74" width="2.7109375" style="4"/>
+    <col min="1" max="2" width="2.6640625" style="6"/>
+    <col min="3" max="3" width="9.33203125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="5.33203125" style="4" customWidth="1"/>
+    <col min="5" max="7" width="2.6640625" style="4"/>
+    <col min="8" max="17" width="2.6640625" style="6"/>
+    <col min="18" max="18" width="7.5546875" style="6" customWidth="1"/>
+    <col min="19" max="46" width="2.6640625" style="6"/>
+    <col min="47" max="47" width="2.6640625" style="6" customWidth="1"/>
+    <col min="48" max="71" width="2.6640625" style="6"/>
+    <col min="72" max="74" width="2.6640625" style="4"/>
     <col min="75" max="75" width="8" style="4" customWidth="1"/>
-    <col min="76" max="76" width="9.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="77" max="16384" width="2.7109375" style="6"/>
+    <col min="76" max="76" width="9.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="77" max="16384" width="2.6640625" style="6"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S3" s="10"/>
       <c r="T3" s="10"/>
       <c r="U3" s="8"/>
@@ -8058,7 +8143,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S4" s="10"/>
       <c r="T4" s="8"/>
       <c r="U4" s="8"/>
@@ -8088,7 +8173,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S5" s="10"/>
       <c r="T5" s="8"/>
       <c r="U5" s="8"/>
@@ -8120,7 +8205,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S6" s="10"/>
       <c r="T6" s="8"/>
       <c r="U6" s="8"/>
@@ -8150,7 +8235,7 @@
       <c r="AP6" s="10"/>
       <c r="AQ6" s="10"/>
     </row>
-    <row r="7" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S7" s="10"/>
       <c r="T7" s="8"/>
       <c r="U7" s="8"/>
@@ -8181,7 +8266,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S8" s="10"/>
       <c r="T8" s="10"/>
       <c r="U8" s="10"/>
@@ -8207,7 +8292,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="9" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S9" s="10"/>
       <c r="T9" s="8"/>
       <c r="U9" s="8"/>
@@ -8233,7 +8318,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S10" s="10"/>
       <c r="T10" s="10"/>
       <c r="U10" s="10"/>
@@ -8260,7 +8345,7 @@
       <c r="AP10" s="10"/>
       <c r="AQ10" s="10"/>
     </row>
-    <row r="11" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="R11" s="6" t="s">
         <v>79</v>
       </c>
@@ -8290,7 +8375,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="12" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="R12" s="6" t="s">
         <v>35</v>
       </c>
@@ -8330,7 +8415,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
@@ -8380,7 +8465,7 @@
       <c r="BW13" s="8"/>
       <c r="BX13" s="8"/>
     </row>
-    <row r="14" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C14" s="8"/>
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
@@ -8430,7 +8515,7 @@
       <c r="BW14" s="8"/>
       <c r="BX14" s="8"/>
     </row>
-    <row r="15" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
@@ -8480,7 +8565,7 @@
       <c r="BW15" s="8"/>
       <c r="BX15" s="8"/>
     </row>
-    <row r="16" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C16" s="8"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
@@ -8524,7 +8609,7 @@
       <c r="BW16" s="8"/>
       <c r="BX16" s="8"/>
     </row>
-    <row r="17" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
@@ -8561,7 +8646,7 @@
       <c r="BW17" s="8"/>
       <c r="BX17" s="8"/>
     </row>
-    <row r="18" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
@@ -8598,7 +8683,7 @@
       <c r="BW18" s="8"/>
       <c r="BX18" s="8"/>
     </row>
-    <row r="19" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C19" s="4" t="s">
         <v>64</v>
       </c>
@@ -8628,7 +8713,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="20" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C20" s="4" t="s">
         <v>60</v>
       </c>
@@ -8659,7 +8744,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="21" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C21" s="4" t="s">
         <v>70</v>
       </c>
@@ -8694,7 +8779,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D22" s="5">
         <v>32</v>
       </c>
@@ -8720,7 +8805,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C23" s="4" t="s">
         <v>66</v>
       </c>
@@ -8752,7 +8837,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="24" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C24" s="4" t="s">
         <v>66</v>
       </c>
@@ -8786,7 +8871,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="25" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C25" s="4" t="s">
         <v>76</v>
       </c>
@@ -8820,7 +8905,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="26" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C26" s="4" t="s">
         <v>66</v>
       </c>
@@ -8850,7 +8935,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="27" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C27" s="4" t="s">
         <v>66</v>
       </c>
@@ -8885,7 +8970,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D28" s="5" t="s">
         <v>53</v>
       </c>
@@ -8914,7 +8999,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="29" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D29" s="5" t="s">
         <v>54</v>
       </c>
@@ -8941,7 +9026,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="30" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D30" s="5" t="s">
         <v>55</v>
       </c>
@@ -8973,7 +9058,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="31" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
       <c r="E31" s="8"/>
@@ -9011,7 +9096,7 @@
       </c>
       <c r="BX31" s="8"/>
     </row>
-    <row r="32" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S32" s="10"/>
       <c r="T32" s="10"/>
       <c r="U32" s="10"/>
@@ -9035,7 +9120,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="33" spans="19:75" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="19:75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S33" s="10"/>
       <c r="T33" s="10"/>
       <c r="U33" s="8"/>
@@ -9059,7 +9144,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="34" spans="19:75" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="19:75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="AL34" s="6" t="s">
         <v>52</v>
       </c>
@@ -9067,9 +9152,9 @@
         <v>59</v>
       </c>
     </row>
-    <row r="41" spans="19:75" ht="15" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="19:75" ht="15" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="19:75" ht="15" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="19:75" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="42" spans="19:75" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="43" spans="19:75" ht="14.4" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -9077,173 +9162,173 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDE3226B-5DED-468C-B710-4E251F22B569}">
   <dimension ref="A1:H25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="1" max="1" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.33203125" customWidth="1"/>
+    <col min="3" max="3" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" t="s">
         <v>100</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>101</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C2" t="s">
         <v>102</v>
       </c>
-      <c r="D1" t="s">
+      <c r="H2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C2" t="s">
-        <v>103</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="B3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D4" s="14" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B3" t="s">
-        <v>103</v>
-      </c>
-      <c r="C3" t="s">
-        <v>103</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>107</v>
-      </c>
-      <c r="B4" t="s">
-        <v>103</v>
-      </c>
-      <c r="C4" t="s">
-        <v>103</v>
-      </c>
-      <c r="D4" s="14" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" t="s">
         <v>110</v>
       </c>
-      <c r="B5" t="s">
-        <v>103</v>
-      </c>
-      <c r="C5" t="s">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C6" t="s">
         <v>112</v>
       </c>
-      <c r="B6" t="s">
-        <v>111</v>
-      </c>
-      <c r="C6" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="F9">
         <v>2.84</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="F10">
         <v>5.75</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="F11">
         <v>8.73</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="F12">
         <v>11.77</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="F13">
         <v>14.88</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="F14">
         <v>18.05</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="F15">
         <v>21.29</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="F16">
         <v>24.59</v>
       </c>
     </row>
-    <row r="17" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F17">
         <v>27.96</v>
       </c>
     </row>
-    <row r="18" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F18">
         <v>31.38</v>
       </c>
     </row>
-    <row r="19" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F19">
         <v>34.869999999999997</v>
       </c>
     </row>
-    <row r="20" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F20">
         <v>38.409999999999997</v>
       </c>
     </row>
-    <row r="21" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F21">
         <v>42.01</v>
       </c>
     </row>
-    <row r="22" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F22">
         <v>45.66</v>
       </c>
     </row>
-    <row r="23" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F23">
         <v>49.36</v>
       </c>
     </row>
-    <row r="24" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F24">
         <v>53.1</v>
       </c>
     </row>
-    <row r="25" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="6:6" x14ac:dyDescent="0.3">
       <c r="F25">
         <v>55</v>
       </c>
@@ -9253,27 +9338,27 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C83C8D3-0A43-41BE-A45D-33BE16890FE8}">
   <dimension ref="C3:BX34"/>
-  <sheetFormatPr defaultColWidth="2.7109375" defaultRowHeight="16.5" thickTop="1" thickBottom="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="2.6640625" defaultRowHeight="15.6" thickTop="1" thickBottom="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="2.7109375" style="6"/>
-    <col min="3" max="3" width="9.28515625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="5.28515625" style="4" customWidth="1"/>
-    <col min="5" max="7" width="2.7109375" style="4"/>
-    <col min="8" max="17" width="2.7109375" style="6"/>
-    <col min="18" max="18" width="7.5703125" style="6" customWidth="1"/>
-    <col min="19" max="46" width="2.7109375" style="6"/>
-    <col min="47" max="47" width="2.7109375" style="6" customWidth="1"/>
-    <col min="48" max="71" width="2.7109375" style="6"/>
-    <col min="72" max="74" width="2.7109375" style="4"/>
+    <col min="1" max="2" width="2.6640625" style="6"/>
+    <col min="3" max="3" width="9.33203125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="5.33203125" style="4" customWidth="1"/>
+    <col min="5" max="7" width="2.6640625" style="4"/>
+    <col min="8" max="17" width="2.6640625" style="6"/>
+    <col min="18" max="18" width="7.5546875" style="6" customWidth="1"/>
+    <col min="19" max="46" width="2.6640625" style="6"/>
+    <col min="47" max="47" width="2.6640625" style="6" customWidth="1"/>
+    <col min="48" max="71" width="2.6640625" style="6"/>
+    <col min="72" max="74" width="2.6640625" style="4"/>
     <col min="75" max="75" width="8" style="4" customWidth="1"/>
-    <col min="76" max="76" width="9.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="77" max="16384" width="2.7109375" style="6"/>
+    <col min="76" max="76" width="9.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="77" max="16384" width="2.6640625" style="6"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S3" s="10"/>
       <c r="T3" s="10"/>
       <c r="U3" s="8"/>
@@ -9296,7 +9381,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S4" s="10"/>
       <c r="T4" s="8"/>
       <c r="U4" s="8"/>
@@ -9326,7 +9411,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S5" s="10"/>
       <c r="T5" s="8"/>
       <c r="U5" s="8"/>
@@ -9358,7 +9443,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S6" s="10"/>
       <c r="T6" s="8"/>
       <c r="U6" s="8"/>
@@ -9388,7 +9473,7 @@
       <c r="AP6" s="10"/>
       <c r="AQ6" s="10"/>
     </row>
-    <row r="7" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S7" s="10"/>
       <c r="T7" s="8"/>
       <c r="U7" s="8"/>
@@ -9419,7 +9504,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S8" s="10"/>
       <c r="T8" s="10"/>
       <c r="U8" s="10"/>
@@ -9445,7 +9530,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="9" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S9" s="10"/>
       <c r="T9" s="8"/>
       <c r="U9" s="8"/>
@@ -9471,7 +9556,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S10" s="10"/>
       <c r="T10" s="10"/>
       <c r="U10" s="10"/>
@@ -9498,7 +9583,7 @@
       <c r="AP10" s="10"/>
       <c r="AQ10" s="10"/>
     </row>
-    <row r="11" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="R11" s="6" t="s">
         <v>79</v>
       </c>
@@ -9528,7 +9613,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="12" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="R12" s="6" t="s">
         <v>35</v>
       </c>
@@ -9568,7 +9653,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
@@ -9618,7 +9703,7 @@
       <c r="BW13" s="8"/>
       <c r="BX13" s="8"/>
     </row>
-    <row r="14" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C14" s="8"/>
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
@@ -9668,7 +9753,7 @@
       <c r="BW14" s="8"/>
       <c r="BX14" s="8"/>
     </row>
-    <row r="15" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
@@ -9718,7 +9803,7 @@
       <c r="BW15" s="8"/>
       <c r="BX15" s="8"/>
     </row>
-    <row r="16" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C16" s="8"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
@@ -9762,7 +9847,7 @@
       <c r="BW16" s="8"/>
       <c r="BX16" s="8"/>
     </row>
-    <row r="17" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
@@ -9799,7 +9884,7 @@
       <c r="BW17" s="8"/>
       <c r="BX17" s="8"/>
     </row>
-    <row r="18" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
@@ -9836,7 +9921,7 @@
       <c r="BW18" s="8"/>
       <c r="BX18" s="8"/>
     </row>
-    <row r="19" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C19" s="4" t="s">
         <v>64</v>
       </c>
@@ -9866,7 +9951,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="20" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C20" s="4" t="s">
         <v>60</v>
       </c>
@@ -9897,7 +9982,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="21" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C21" s="4" t="s">
         <v>70</v>
       </c>
@@ -9932,7 +10017,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D22" s="5">
         <v>32</v>
       </c>
@@ -9958,7 +10043,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C23" s="4" t="s">
         <v>66</v>
       </c>
@@ -9990,7 +10075,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="24" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C24" s="4" t="s">
         <v>66</v>
       </c>
@@ -10024,7 +10109,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="25" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C25" s="4" t="s">
         <v>76</v>
       </c>
@@ -10058,7 +10143,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="26" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C26" s="4" t="s">
         <v>66</v>
       </c>
@@ -10088,7 +10173,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="27" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C27" s="4" t="s">
         <v>66</v>
       </c>
@@ -10123,7 +10208,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D28" s="5" t="s">
         <v>53</v>
       </c>
@@ -10152,7 +10237,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="29" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D29" s="5" t="s">
         <v>54</v>
       </c>
@@ -10179,7 +10264,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="30" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D30" s="5" t="s">
         <v>55</v>
       </c>
@@ -10211,7 +10296,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="31" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
       <c r="E31" s="8"/>
@@ -10249,7 +10334,7 @@
       </c>
       <c r="BX31" s="8"/>
     </row>
-    <row r="32" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:76" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S32" s="10"/>
       <c r="T32" s="10"/>
       <c r="U32" s="10"/>
@@ -10273,7 +10358,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="33" spans="19:75" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="19:75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="S33" s="10"/>
       <c r="T33" s="10"/>
       <c r="U33" s="8"/>
@@ -10297,7 +10382,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="34" spans="19:75" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="19:75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="AL34" s="6" t="s">
         <v>52</v>
       </c>

</xml_diff>

<commit_message>
Fix preprocessing pipeline so it works with zeroing disabled. CHange interpretation of schematic roles so ops not indicated are allowed. Change segment and event extraction to use registry for roles.
</commit_message>
<xml_diff>
--- a/To do/To do list.xlsx
+++ b/To do/To do list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benco\dev\BODAQS\To do\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94877A1A-BA37-4118-87CB-090657EE4E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{549FC000-CECA-464A-A16D-56C58FDC960E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="186">
   <si>
     <t>Requirements</t>
   </si>
@@ -574,21 +574,12 @@
     <t>Pass activity-mask parameters from notebook</t>
   </si>
   <si>
-    <t>Pre-processing fails if zeroing is false</t>
-  </si>
-  <si>
     <t>Widgets - option to display sessions by description</t>
   </si>
   <si>
-    <t>Signal histogram widget: more elaborate detection of available signals</t>
-  </si>
-  <si>
     <t>Download all / delete all</t>
   </si>
   <si>
-    <t>Tidy up session window</t>
-  </si>
-  <si>
     <t>Iterate event schema - all the events</t>
   </si>
   <si>
@@ -604,13 +595,13 @@
     <t>rear</t>
   </si>
   <si>
-    <t>Don't zero in place</t>
-  </si>
-  <si>
     <t>Pass zeroing parameters dynamically</t>
   </si>
   <si>
     <t>Test clipping</t>
+  </si>
+  <si>
+    <t>SAMPLE_RATE_HZ = 500   # if known; used for VA estimation when time col is absent - drop this</t>
   </si>
 </sst>
 </file>
@@ -7552,48 +7543,34 @@
         <v>118</v>
       </c>
       <c r="C36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>119</v>
       </c>
-      <c r="C37" t="s">
-        <v>178</v>
-      </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>153</v>
       </c>
       <c r="C40" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
-      <c r="C41" t="s">
-        <v>181</v>
-      </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="16" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C43" t="s">
-        <v>176</v>
-      </c>
-    </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>131</v>
       </c>
-      <c r="C44" t="s">
-        <v>186</v>
-      </c>
       <c r="E44" t="s">
         <v>126</v>
       </c>
@@ -7603,7 +7580,7 @@
         <v>132</v>
       </c>
       <c r="C45" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="E45" t="s">
         <v>127</v>
@@ -7622,7 +7599,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C47" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
@@ -7634,6 +7611,9 @@
       <c r="A50" t="s">
         <v>152</v>
       </c>
+      <c r="C50" t="s">
+        <v>185</v>
+      </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
@@ -7735,12 +7715,12 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -7756,12 +7736,12 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B2">
         <v>3433</v>
@@ -7769,7 +7749,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B3">
         <v>3564</v>

</xml_diff>

<commit_message>
Move to VSCode / PlatformIO for firmware development and install VSCode Codex extension. Test build and resolve build issues.
</commit_message>
<xml_diff>
--- a/To do/To do list.xlsx
+++ b/To do/To do list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benco\dev\BODAQS\To do\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{549FC000-CECA-464A-A16D-56C58FDC960E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9591DB51-4AC1-4DEF-A2F4-64EB2B9F76F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="185">
   <si>
     <t>Requirements</t>
   </si>
@@ -409,9 +409,6 @@
     <t>Mechanical</t>
   </si>
   <si>
-    <t>Design for stripboard version</t>
-  </si>
-  <si>
     <t>Add power management</t>
   </si>
   <si>
@@ -424,9 +421,6 @@
     <t>Sensor re-factor and individual sample rate</t>
   </si>
   <si>
-    <t>2 channel + I2C stripboard through-hole</t>
-  </si>
-  <si>
     <t>4 channel + I2C PCB through-hole, with UI and without</t>
   </si>
   <si>
@@ -571,15 +565,9 @@
     <t>Domains derived from some master source</t>
   </si>
   <si>
-    <t>Pass activity-mask parameters from notebook</t>
-  </si>
-  <si>
     <t>Widgets - option to display sessions by description</t>
   </si>
   <si>
-    <t>Download all / delete all</t>
-  </si>
-  <si>
     <t>Iterate event schema - all the events</t>
   </si>
   <si>
@@ -595,13 +583,22 @@
     <t>rear</t>
   </si>
   <si>
-    <t>Pass zeroing parameters dynamically</t>
-  </si>
-  <si>
     <t>Test clipping</t>
   </si>
   <si>
-    <t>SAMPLE_RATE_HZ = 500   # if known; used for VA estimation when time col is absent - drop this</t>
+    <t>VA - just run on displacement columns</t>
+  </si>
+  <si>
+    <t>activity mask preview</t>
+  </si>
+  <si>
+    <t>zeroing preview</t>
+  </si>
+  <si>
+    <t>Logger semantics dictionary</t>
+  </si>
+  <si>
+    <t>Widgets - statistics</t>
   </si>
 </sst>
 </file>
@@ -7296,9 +7293,9 @@
   <dimension ref="A1:G75"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.5546875" customWidth="1"/>
-    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="3" max="3" width="64.5546875" customWidth="1"/>
     <col min="5" max="5" width="39.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7488,16 +7485,13 @@
       <c r="C29" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="E29" t="s">
-        <v>121</v>
-      </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>95</v>
       </c>
       <c r="E30" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
@@ -7505,7 +7499,7 @@
         <v>96</v>
       </c>
       <c r="E31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
@@ -7515,18 +7509,18 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E33" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E34" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
@@ -7535,16 +7529,13 @@
       </c>
       <c r="C35" s="1"/>
       <c r="E35" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>118</v>
       </c>
-      <c r="C36" t="s">
-        <v>176</v>
-      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
@@ -7553,10 +7544,10 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>153</v>
-      </c>
-      <c r="C40" t="s">
-        <v>178</v>
+        <v>151</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
@@ -7564,163 +7555,161 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="16" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>131</v>
-      </c>
-      <c r="E44" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>132</v>
-      </c>
-      <c r="C45" t="s">
-        <v>183</v>
+        <v>130</v>
       </c>
       <c r="E45" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>133</v>
-      </c>
-      <c r="C46" t="s">
-        <v>175</v>
+        <v>131</v>
       </c>
       <c r="E46" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C47" t="s">
-        <v>184</v>
+        <v>126</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="13" t="s">
-        <v>135</v>
+        <v>133</v>
+      </c>
+      <c r="C48" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C49" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C50" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
+      </c>
+      <c r="C51" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>169</v>
+        <v>167</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>170</v>
+        <v>168</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C54" s="3" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="13" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C61" s="1"/>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C62" s="1"/>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C63" s="1"/>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>163</v>
-      </c>
-      <c r="C65" s="1"/>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C66" s="1"/>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
         <v>171</v>
       </c>
-      <c r="C67" s="1"/>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A71" s="3" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A70" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A75" t="s">
-        <v>179</v>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A75" s="3" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -7736,12 +7725,12 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B2">
         <v>3433</v>
@@ -7749,7 +7738,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B3">
         <v>3564</v>
@@ -7818,10 +7807,10 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -7988,21 +7977,21 @@
   <sheetData>
     <row r="4" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E4" t="s">
+        <v>136</v>
+      </c>
+      <c r="G4" t="s">
+        <v>137</v>
+      </c>
+      <c r="I4" t="s">
         <v>138</v>
-      </c>
-      <c r="G4" t="s">
-        <v>139</v>
-      </c>
-      <c r="I4" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="5" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F5" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -8011,13 +8000,13 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="M5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="5:13" x14ac:dyDescent="0.3">
@@ -8025,7 +8014,7 @@
         <v>70</v>
       </c>
       <c r="F6" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G6">
         <v>2</v>
@@ -8034,18 +8023,18 @@
         <v>2</v>
       </c>
       <c r="J6" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="L6" t="s">
+        <v>142</v>
+      </c>
+      <c r="M6" t="s">
         <v>144</v>
-      </c>
-      <c r="M6" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="7" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F7" t="s">
         <v>83</v>
@@ -8057,21 +8046,21 @@
         <v>3</v>
       </c>
       <c r="J7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="L7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="M7" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="5:13" x14ac:dyDescent="0.3">
       <c r="L8" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="M8" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add a test harness notebook for developing event definitions
</commit_message>
<xml_diff>
--- a/To do/To do list.xlsx
+++ b/To do/To do list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benco\dev\BODAQS\To do\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9591DB51-4AC1-4DEF-A2F4-64EB2B9F76F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{369D1F94-B290-48BA-A5D3-DF1302057A5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
   </bookViews>
@@ -7593,7 +7593,7 @@
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
+      <c r="A50" s="1" t="s">
         <v>150</v>
       </c>
       <c r="C50" t="s">
@@ -7609,7 +7609,7 @@
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
+      <c r="A52" s="1" t="s">
         <v>167</v>
       </c>
       <c r="C52" s="3" t="s">
@@ -7708,7 +7708,7 @@
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A75" s="3" t="s">
+      <c r="A75" s="1" t="s">
         <v>175</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Polish run library formatting and behaviour
</commit_message>
<xml_diff>
--- a/To do/To do list.xlsx
+++ b/To do/To do list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benco\dev\BODAQS\To do\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{369D1F94-B290-48BA-A5D3-DF1302057A5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6D405C5-9DD0-46D7-A160-B4068094364C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
   </bookViews>
@@ -24,6 +24,7 @@
     <sheet name="Stripboard (2)" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="183">
   <si>
     <t>Requirements</t>
   </si>
@@ -565,9 +566,6 @@
     <t>Domains derived from some master source</t>
   </si>
   <si>
-    <t>Widgets - option to display sessions by description</t>
-  </si>
-  <si>
     <t>Iterate event schema - all the events</t>
   </si>
   <si>
@@ -586,19 +584,16 @@
     <t>Test clipping</t>
   </si>
   <si>
-    <t>VA - just run on displacement columns</t>
-  </si>
-  <si>
-    <t>activity mask preview</t>
-  </si>
-  <si>
-    <t>zeroing preview</t>
-  </si>
-  <si>
-    <t>Logger semantics dictionary</t>
-  </si>
-  <si>
-    <t>Widgets - statistics</t>
+    <t>Tidy up basic event detection</t>
+  </si>
+  <si>
+    <t>Preprocessing - add lineage to registry</t>
+  </si>
+  <si>
+    <t>Add secondary sensor to event browser</t>
+  </si>
+  <si>
+    <t>Event test harness fix</t>
   </si>
 </sst>
 </file>
@@ -7547,7 +7542,7 @@
         <v>151</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
@@ -7584,49 +7579,32 @@
         <v>133</v>
       </c>
       <c r="C48" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C49" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="C50" t="s">
-        <v>181</v>
-      </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C51" t="s">
-        <v>182</v>
-      </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="C52" s="3" t="s">
-        <v>183</v>
-      </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>168</v>
       </c>
-      <c r="C53" s="3" t="s">
-        <v>173</v>
-      </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C54" s="3" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
@@ -7648,6 +7626,9 @@
       <c r="A58" t="s">
         <v>155</v>
       </c>
+      <c r="C58" s="3" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
@@ -7658,12 +7639,17 @@
       <c r="A60" t="s">
         <v>157</v>
       </c>
+      <c r="C60" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>158</v>
       </c>
-      <c r="C61" s="1"/>
+      <c r="C61" t="s">
+        <v>182</v>
+      </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
@@ -7709,7 +7695,7 @@
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -7725,12 +7711,12 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B2">
         <v>3433</v>
@@ -7738,7 +7724,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B3">
         <v>3564</v>

</xml_diff>

<commit_message>
Investigate issues with as5600 on I2C
</commit_message>
<xml_diff>
--- a/To do/To do list.xlsx
+++ b/To do/To do list.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benco\dev\BODAQS\To do\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6D405C5-9DD0-46D7-A160-B4068094364C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C02AB46-8606-460E-B9CD-1B4F76186319}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{50899B05-5FED-46D9-9A48-93F2B68E0E6B}"/>
   </bookViews>
@@ -24,7 +24,6 @@
     <sheet name="Stripboard (2)" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -7652,7 +7651,7 @@
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
+      <c r="A62" s="1" t="s">
         <v>159</v>
       </c>
       <c r="C62" s="1"/>

</xml_diff>